<commit_message>
extration FC sur HAL + modif affichages
</commit_message>
<xml_diff>
--- a/Data/FairCarboN_Datas_Contacts2.xlsx
+++ b/Data/FairCarboN_Datas_Contacts2.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dutroncj\Documents\Outils\FairCarboN_datas\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C0AE0AA-DD4B-489E-BA3B-8970B9DF52E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8290BB28-EAC7-4056-A354-9922EEFF9C4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Liste" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Liste!$A$1:$B$566</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Liste!$A$1:$B$564</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1132" uniqueCount="524">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1128" uniqueCount="524">
   <si>
     <t>ALAMOD</t>
   </si>
@@ -1428,9 +1428,6 @@
     <t xml:space="preserve"> Guillaume Bertrand</t>
   </si>
   <si>
-    <t>Carbonium</t>
-  </si>
-  <si>
     <t>Eléa Frétigné</t>
   </si>
   <si>
@@ -1452,12 +1449,6 @@
     <t>Marttiina Rentala</t>
   </si>
   <si>
-    <t>Deepc</t>
-  </si>
-  <si>
-    <t>tropecos</t>
-  </si>
-  <si>
     <t>François Gevaert</t>
   </si>
   <si>
@@ -1497,9 +1488,6 @@
     <t>Claire Cénac</t>
   </si>
   <si>
-    <t>cabestan</t>
-  </si>
-  <si>
     <t>Marie  Alexis</t>
   </si>
   <si>
@@ -1518,9 +1506,6 @@
     <t>César CIEBIERA</t>
   </si>
   <si>
-    <t>Peace</t>
-  </si>
-  <si>
     <t>Kamel Elouhichi</t>
   </si>
   <si>
@@ -1542,21 +1527,12 @@
     <t xml:space="preserve">Philippe Peylin </t>
   </si>
   <si>
-    <t>climfas</t>
-  </si>
-  <si>
-    <t>prefalim</t>
-  </si>
-  <si>
     <t>Isabelle Basile-Doelsch</t>
   </si>
   <si>
     <t>Puu Tai Yang</t>
   </si>
   <si>
-    <t>rhizoseqc</t>
-  </si>
-  <si>
     <t>Sixteen Cueff</t>
   </si>
   <si>
@@ -1566,9 +1542,6 @@
     <t>Maelle Pomies</t>
   </si>
   <si>
-    <t>canete</t>
-  </si>
-  <si>
     <t>Véronique Receveur-Brechot</t>
   </si>
   <si>
@@ -1590,25 +1563,52 @@
     <t>Hirono Suzuki</t>
   </si>
   <si>
-    <t>co2cmphi</t>
-  </si>
-  <si>
     <t>Mathias Cuntz</t>
   </si>
   <si>
-    <t>droughtforc</t>
-  </si>
-  <si>
     <t>Antoine Fournier</t>
   </si>
   <si>
     <t>Benjamin Gac</t>
   </si>
   <si>
-    <t>greenscale</t>
-  </si>
-  <si>
     <t>CrosyeN</t>
+  </si>
+  <si>
+    <t>CABESTAN</t>
+  </si>
+  <si>
+    <t>CANETE</t>
+  </si>
+  <si>
+    <t>CarboNium</t>
+  </si>
+  <si>
+    <t>CLIM-FAS</t>
+  </si>
+  <si>
+    <t>CO2_CMPhi</t>
+  </si>
+  <si>
+    <t>DEEP-C</t>
+  </si>
+  <si>
+    <t>DroughtForC</t>
+  </si>
+  <si>
+    <t>GREENSCALE</t>
+  </si>
+  <si>
+    <t>PEACE</t>
+  </si>
+  <si>
+    <t>PREFALIM</t>
+  </si>
+  <si>
+    <t>RhizoSeqC</t>
+  </si>
+  <si>
+    <t>TROPECOS</t>
   </si>
 </sst>
 </file>
@@ -1980,7 +1980,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:B566"/>
+  <dimension ref="A1:B564"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.453125" style="2" bestFit="1" customWidth="1"/>
@@ -2910,7 +2910,7 @@
     </row>
     <row r="116" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B116" s="5" t="s">
         <v>81</v>
@@ -2918,7 +2918,7 @@
     </row>
     <row r="117" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B117" s="5" t="s">
         <v>315</v>
@@ -2926,7 +2926,7 @@
     </row>
     <row r="118" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B118" s="5" t="s">
         <v>316</v>
@@ -2934,7 +2934,7 @@
     </row>
     <row r="119" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B119" s="5" t="s">
         <v>231</v>
@@ -2942,7 +2942,7 @@
     </row>
     <row r="120" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B120" s="5" t="s">
         <v>317</v>
@@ -2950,7 +2950,7 @@
     </row>
     <row r="121" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B121" s="5" t="s">
         <v>228</v>
@@ -2958,7 +2958,7 @@
     </row>
     <row r="122" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B122" s="5" t="s">
         <v>318</v>
@@ -2966,7 +2966,7 @@
     </row>
     <row r="123" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B123" s="5" t="s">
         <v>319</v>
@@ -2974,7 +2974,7 @@
     </row>
     <row r="124" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B124" s="5" t="s">
         <v>320</v>
@@ -2982,7 +2982,7 @@
     </row>
     <row r="125" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B125" s="5" t="s">
         <v>321</v>
@@ -2990,7 +2990,7 @@
     </row>
     <row r="126" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B126" s="5" t="s">
         <v>322</v>
@@ -2998,7 +2998,7 @@
     </row>
     <row r="127" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B127" s="5" t="s">
         <v>323</v>
@@ -3006,7 +3006,7 @@
     </row>
     <row r="128" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B128" s="5" t="s">
         <v>324</v>
@@ -3014,7 +3014,7 @@
     </row>
     <row r="129" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B129" s="5" t="s">
         <v>325</v>
@@ -3022,7 +3022,7 @@
     </row>
     <row r="130" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A130" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B130" s="5" t="s">
         <v>47</v>
@@ -3030,7 +3030,7 @@
     </row>
     <row r="131" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A131" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B131" s="5" t="s">
         <v>326</v>
@@ -3038,7 +3038,7 @@
     </row>
     <row r="132" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A132" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B132" s="5" t="s">
         <v>72</v>
@@ -3046,7 +3046,7 @@
     </row>
     <row r="133" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B133" s="5" t="s">
         <v>395</v>
@@ -3054,7 +3054,7 @@
     </row>
     <row r="134" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A134" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B134" s="5" t="s">
         <v>327</v>
@@ -3062,7 +3062,7 @@
     </row>
     <row r="135" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A135" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B135" s="5" t="s">
         <v>217</v>
@@ -3070,7 +3070,7 @@
     </row>
     <row r="136" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B136" s="5" t="s">
         <v>328</v>
@@ -3078,7 +3078,7 @@
     </row>
     <row r="137" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B137" s="5" t="s">
         <v>461</v>
@@ -3086,7 +3086,7 @@
     </row>
     <row r="138" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A138" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B138" s="5" t="s">
         <v>329</v>
@@ -3094,7 +3094,7 @@
     </row>
     <row r="139" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A139" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B139" s="5" t="s">
         <v>330</v>
@@ -3102,7 +3102,7 @@
     </row>
     <row r="140" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A140" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B140" s="5" t="s">
         <v>331</v>
@@ -3110,7 +3110,7 @@
     </row>
     <row r="141" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A141" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B141" s="5" t="s">
         <v>332</v>
@@ -3118,7 +3118,7 @@
     </row>
     <row r="142" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A142" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B142" s="5" t="s">
         <v>333</v>
@@ -3126,7 +3126,7 @@
     </row>
     <row r="143" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A143" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B143" s="5" t="s">
         <v>334</v>
@@ -3134,7 +3134,7 @@
     </row>
     <row r="144" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A144" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B144" s="5" t="s">
         <v>342</v>
@@ -3142,7 +3142,7 @@
     </row>
     <row r="145" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A145" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B145" s="5" t="s">
         <v>335</v>
@@ -3150,7 +3150,7 @@
     </row>
     <row r="146" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A146" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B146" s="5" t="s">
         <v>48</v>
@@ -3158,7 +3158,7 @@
     </row>
     <row r="147" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A147" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B147" s="5" t="s">
         <v>230</v>
@@ -3166,7 +3166,7 @@
     </row>
     <row r="148" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A148" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B148" s="5" t="s">
         <v>49</v>
@@ -3174,7 +3174,7 @@
     </row>
     <row r="149" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A149" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B149" s="5" t="s">
         <v>336</v>
@@ -3182,7 +3182,7 @@
     </row>
     <row r="150" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A150" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B150" s="5" t="s">
         <v>361</v>
@@ -3190,7 +3190,7 @@
     </row>
     <row r="151" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A151" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B151" s="5" t="s">
         <v>372</v>
@@ -3198,7 +3198,7 @@
     </row>
     <row r="152" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A152" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B152" s="5" t="s">
         <v>384</v>
@@ -3206,7 +3206,7 @@
     </row>
     <row r="153" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A153" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B153" s="5" t="s">
         <v>385</v>
@@ -3214,7 +3214,7 @@
     </row>
     <row r="154" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A154" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B154" s="5" t="s">
         <v>202</v>
@@ -3222,7 +3222,7 @@
     </row>
     <row r="155" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A155" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B155" s="5" t="s">
         <v>396</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="156" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A156" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B156" s="5" t="s">
         <v>397</v>
@@ -3238,7 +3238,7 @@
     </row>
     <row r="157" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A157" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B157" s="5" t="s">
         <v>462</v>
@@ -3246,7 +3246,7 @@
     </row>
     <row r="158" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A158" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B158" s="5" t="s">
         <v>398</v>
@@ -3254,7 +3254,7 @@
     </row>
     <row r="159" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A159" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B159" s="5" t="s">
         <v>399</v>
@@ -3262,7 +3262,7 @@
     </row>
     <row r="160" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A160" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B160" s="5" t="s">
         <v>400</v>
@@ -3270,7 +3270,7 @@
     </row>
     <row r="161" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A161" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B161" s="5" t="s">
         <v>401</v>
@@ -3278,7 +3278,7 @@
     </row>
     <row r="162" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A162" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B162" s="5" t="s">
         <v>402</v>
@@ -3286,7 +3286,7 @@
     </row>
     <row r="163" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A163" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B163" s="5" t="s">
         <v>403</v>
@@ -3294,7 +3294,7 @@
     </row>
     <row r="164" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A164" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B164" s="5" t="s">
         <v>404</v>
@@ -3302,7 +3302,7 @@
     </row>
     <row r="165" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A165" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B165" s="5" t="s">
         <v>405</v>
@@ -3310,7 +3310,7 @@
     </row>
     <row r="166" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A166" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B166" s="5" t="s">
         <v>406</v>
@@ -3318,7 +3318,7 @@
     </row>
     <row r="167" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A167" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B167" s="5" t="s">
         <v>407</v>
@@ -3326,7 +3326,7 @@
     </row>
     <row r="168" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A168" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B168" s="5" t="s">
         <v>408</v>
@@ -3334,7 +3334,7 @@
     </row>
     <row r="169" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A169" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B169" s="5" t="s">
         <v>409</v>
@@ -3342,7 +3342,7 @@
     </row>
     <row r="170" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A170" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B170" s="5" t="s">
         <v>410</v>
@@ -3350,7 +3350,7 @@
     </row>
     <row r="171" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A171" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B171" s="5" t="s">
         <v>411</v>
@@ -3358,7 +3358,7 @@
     </row>
     <row r="172" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A172" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B172" s="5" t="s">
         <v>412</v>
@@ -3366,7 +3366,7 @@
     </row>
     <row r="173" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A173" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B173" s="5" t="s">
         <v>314</v>
@@ -3374,7 +3374,7 @@
     </row>
     <row r="174" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A174" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B174" s="5" t="s">
         <v>71</v>
@@ -3382,7 +3382,7 @@
     </row>
     <row r="175" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A175" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B175" s="5" t="s">
         <v>73</v>
@@ -3390,7 +3390,7 @@
     </row>
     <row r="176" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A176" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B176" s="5" t="s">
         <v>55</v>
@@ -3398,7 +3398,7 @@
     </row>
     <row r="177" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A177" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B177" s="5" t="s">
         <v>80</v>
@@ -3406,7 +3406,7 @@
     </row>
     <row r="178" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A178" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B178" s="5" t="s">
         <v>52</v>
@@ -3414,7 +3414,7 @@
     </row>
     <row r="179" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A179" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B179" s="5" t="s">
         <v>216</v>
@@ -3422,7 +3422,7 @@
     </row>
     <row r="180" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A180" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B180" s="5" t="s">
         <v>413</v>
@@ -3430,7 +3430,7 @@
     </row>
     <row r="181" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A181" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B181" s="5" t="s">
         <v>68</v>
@@ -3438,7 +3438,7 @@
     </row>
     <row r="182" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A182" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B182" s="5" t="s">
         <v>197</v>
@@ -3446,7 +3446,7 @@
     </row>
     <row r="183" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A183" s="1" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="B183" s="5" t="s">
         <v>236</v>
@@ -3454,314 +3454,314 @@
     </row>
     <row r="184" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A184" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B184" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A185" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B185" s="5" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A186" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B186" s="5" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A187" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B187" s="5" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A188" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B188" s="5" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A189" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B189" s="5" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A190" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B190" s="5" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A191" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B191" s="5" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A192" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B192" s="5" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A193" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B193" s="5" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A194" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B194" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A195" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B195" s="5" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A196" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B196" s="5" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A197" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B197" s="5" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A198" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B198" s="5" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A199" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B199" s="5" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A200" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B200" s="5" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A201" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B201" s="5" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A202" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B202" s="5" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A203" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B203" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A204" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B204" s="5" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A205" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B205" s="5" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A206" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B206" s="5" t="s">
         <v>463</v>
       </c>
-      <c r="B184" s="5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="185" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A185" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B185" s="5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="186" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A186" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B186" s="5" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="187" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A187" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B187" s="5" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="188" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A188" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B188" s="5" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="189" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A189" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B189" s="5" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="190" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A190" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B190" s="5" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="191" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A191" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B191" s="5" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="192" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A192" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B192" s="5" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="193" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A193" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B193" s="5" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="194" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A194" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B194" s="5" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="195" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A195" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B195" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="196" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A196" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B196" s="5" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="197" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A197" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B197" s="5" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="198" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A198" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B198" s="5" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="199" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A199" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B199" s="5" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="200" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A200" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B200" s="5" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="201" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A201" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B201" s="5" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="202" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A202" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B202" s="5" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="203" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A203" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B203" s="5" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="204" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A204" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B204" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="205" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A205" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B205" s="5" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="206" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A206" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B206" s="5" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="207" spans="1:2" x14ac:dyDescent="0.35">
+    </row>
+    <row r="207" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A207" s="1" t="s">
-        <v>523</v>
+        <v>511</v>
       </c>
       <c r="B207" s="5" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A208" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B208" s="5" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A209" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B209" s="5" t="s">
         <v>464</v>
       </c>
     </row>
-    <row r="208" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A208" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B208" s="5" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="209" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A209" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B209" s="5" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="210" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A210" s="1" t="s">
-        <v>523</v>
+        <v>511</v>
       </c>
       <c r="B210" s="5" t="s">
         <v>465</v>
       </c>
     </row>
-    <row r="211" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A211" s="1" t="s">
-        <v>523</v>
+        <v>511</v>
       </c>
       <c r="B211" s="5" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A212" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B212" s="5" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A213" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B213" s="5" t="s">
         <v>466</v>
       </c>
     </row>
-    <row r="212" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A212" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B212" s="5" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="213" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A213" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B213" s="5" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="214" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A214" s="1" t="s">
-        <v>523</v>
+        <v>511</v>
       </c>
       <c r="B214" s="5" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A215" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B215" s="5" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A216" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B216" s="5" t="s">
         <v>467</v>
       </c>
     </row>
-    <row r="215" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A215" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B215" s="5" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="216" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A216" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B216" s="5" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="217" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A217" s="1" t="s">
-        <v>523</v>
+        <v>511</v>
       </c>
       <c r="B217" s="5" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="218" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A218" s="1" t="s">
-        <v>523</v>
+        <v>511</v>
       </c>
       <c r="B218" s="5" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="219" spans="1:2" x14ac:dyDescent="0.35">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A219" s="1" t="s">
-        <v>523</v>
+        <v>511</v>
       </c>
       <c r="B219" s="5" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="220" spans="1:2" x14ac:dyDescent="0.35">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A220" s="1" t="s">
-        <v>523</v>
+        <v>511</v>
       </c>
       <c r="B220" s="5" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="221" spans="1:2" x14ac:dyDescent="0.35">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A221" s="1" t="s">
-        <v>523</v>
+        <v>511</v>
       </c>
       <c r="B221" s="5" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="222" spans="1:2" x14ac:dyDescent="0.35">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A222" s="1" t="s">
-        <v>523</v>
+        <v>2</v>
       </c>
       <c r="B222" s="5" t="s">
-        <v>426</v>
+        <v>4</v>
       </c>
     </row>
     <row r="223" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
@@ -3769,7 +3769,7 @@
         <v>2</v>
       </c>
       <c r="B223" s="5" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="224" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
@@ -3777,7 +3777,7 @@
         <v>2</v>
       </c>
       <c r="B224" s="5" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="225" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
@@ -3785,7 +3785,7 @@
         <v>2</v>
       </c>
       <c r="B225" s="5" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="226" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
@@ -3793,7 +3793,7 @@
         <v>2</v>
       </c>
       <c r="B226" s="5" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="227" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
@@ -3801,7 +3801,7 @@
         <v>2</v>
       </c>
       <c r="B227" s="5" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="228" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
@@ -3809,7 +3809,7 @@
         <v>2</v>
       </c>
       <c r="B228" s="5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="229" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
@@ -3817,7 +3817,7 @@
         <v>2</v>
       </c>
       <c r="B229" s="5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="230" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
@@ -3825,7 +3825,7 @@
         <v>2</v>
       </c>
       <c r="B230" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="231" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
@@ -3833,7 +3833,7 @@
         <v>2</v>
       </c>
       <c r="B231" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="232" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
@@ -3841,7 +3841,7 @@
         <v>2</v>
       </c>
       <c r="B232" s="5" t="s">
-        <v>12</v>
+        <v>191</v>
       </c>
     </row>
     <row r="233" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
@@ -3849,7 +3849,7 @@
         <v>2</v>
       </c>
       <c r="B233" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="234" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
@@ -3857,7 +3857,7 @@
         <v>2</v>
       </c>
       <c r="B234" s="5" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="235" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
@@ -3865,7 +3865,7 @@
         <v>2</v>
       </c>
       <c r="B235" s="5" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="236" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
@@ -3873,7 +3873,7 @@
         <v>2</v>
       </c>
       <c r="B236" s="5" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="237" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
@@ -3881,7 +3881,7 @@
         <v>2</v>
       </c>
       <c r="B237" s="5" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="238" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
@@ -3889,7 +3889,7 @@
         <v>2</v>
       </c>
       <c r="B238" s="5" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="239" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
@@ -3897,2439 +3897,2439 @@
         <v>2</v>
       </c>
       <c r="B239" s="5" t="s">
-        <v>197</v>
+        <v>391</v>
       </c>
     </row>
     <row r="240" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A240" s="1" t="s">
-        <v>2</v>
+        <v>517</v>
       </c>
       <c r="B240" s="5" t="s">
-        <v>391</v>
+        <v>5</v>
       </c>
     </row>
     <row r="241" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A241" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B241" s="5" t="s">
-        <v>5</v>
+        <v>41</v>
       </c>
     </row>
     <row r="242" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A242" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B242" s="5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="243" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A243" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B243" s="5" t="s">
-        <v>43</v>
+        <v>469</v>
       </c>
     </row>
     <row r="244" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A244" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B244" s="5" t="s">
-        <v>470</v>
+        <v>42</v>
       </c>
     </row>
     <row r="245" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A245" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B245" s="5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="246" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A246" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B246" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="247" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A247" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B247" s="5" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
     </row>
     <row r="248" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A248" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B248" s="5" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
     </row>
     <row r="249" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A249" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B249" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="250" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A250" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B250" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="251" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A251" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B251" s="5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="252" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A252" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B252" s="5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="253" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A253" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B253" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="254" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A254" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B254" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="255" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A255" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B255" s="5" t="s">
-        <v>52</v>
+        <v>73</v>
       </c>
     </row>
     <row r="256" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A256" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B256" s="5" t="s">
-        <v>73</v>
+        <v>53</v>
       </c>
     </row>
     <row r="257" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A257" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B257" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="258" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A258" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B258" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="259" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A259" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B259" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="260" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A260" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B260" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="261" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A261" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B261" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="262" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A262" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B262" s="5" t="s">
-        <v>58</v>
+        <v>340</v>
       </c>
     </row>
     <row r="263" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A263" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B263" s="5" t="s">
-        <v>340</v>
+        <v>59</v>
       </c>
     </row>
     <row r="264" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A264" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B264" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="265" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A265" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B265" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="266" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A266" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B266" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="267" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A267" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B267" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="268" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A268" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B268" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="269" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A269" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B269" s="5" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
     </row>
     <row r="270" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A270" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B270" s="5" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
     </row>
     <row r="271" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A271" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B271" s="5" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
     </row>
     <row r="272" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A272" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B272" s="5" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
     </row>
     <row r="273" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A273" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B273" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="274" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A274" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B274" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="275" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A275" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B275" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="276" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A276" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B276" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="277" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A277" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B277" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="278" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A278" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B278" s="5" t="s">
-        <v>71</v>
+        <v>380</v>
       </c>
     </row>
     <row r="279" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A279" s="1" t="s">
-        <v>471</v>
+        <v>517</v>
       </c>
       <c r="B279" s="5" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="280" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="280" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A280" s="1" t="s">
-        <v>471</v>
+        <v>523</v>
       </c>
       <c r="B280" s="5" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="281" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="281" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A281" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B281" s="5" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="282" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="282" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A282" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B282" s="5" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="283" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="283" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A283" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B283" s="5" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="284" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="284" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A284" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B284" s="5" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="285" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="285" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A285" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B285" s="5" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="286" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="286" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A286" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B286" s="5" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="287" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="287" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A287" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B287" s="5" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="288" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="288" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A288" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B288" s="5" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="289" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="289" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A289" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B289" s="5" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="290" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="290" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A290" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B290" s="5" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="291" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="291" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A291" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B291" s="5" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="292" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="292" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A292" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B292" s="5" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="293" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="293" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A293" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B293" s="5" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="294" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="294" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A294" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B294" s="5" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="295" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="295" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A295" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B295" s="5" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="296" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="296" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A296" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B296" s="5" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="297" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="297" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A297" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B297" s="5" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="298" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="298" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A298" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B298" s="5" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="299" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="299" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A299" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B299" s="5" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="300" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="300" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A300" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B300" s="5" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="301" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="301" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A301" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B301" s="5" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="302" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="302" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A302" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B302" s="5" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="303" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="303" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A303" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B303" s="5" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="304" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="304" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A304" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B304" s="5" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="305" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="305" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A305" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B305" s="5" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="306" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="306" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A306" s="1" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="B306" s="5" t="s">
-        <v>363</v>
+        <v>373</v>
       </c>
     </row>
     <row r="307" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A307" s="1" t="s">
-        <v>472</v>
+        <v>512</v>
       </c>
       <c r="B307" s="5" t="s">
-        <v>373</v>
+        <v>224</v>
       </c>
     </row>
     <row r="308" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A308" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B308" s="5" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
     </row>
     <row r="309" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A309" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B309" s="5" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="310" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A310" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B310" s="5" t="s">
-        <v>236</v>
+        <v>225</v>
       </c>
     </row>
     <row r="311" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A311" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B311" s="5" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="312" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A312" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B312" s="5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="313" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A313" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B313" s="5" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="314" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A314" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B314" s="5" t="s">
-        <v>228</v>
+        <v>217</v>
       </c>
     </row>
     <row r="315" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A315" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B315" s="5" t="s">
-        <v>217</v>
+        <v>229</v>
       </c>
     </row>
     <row r="316" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A316" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B316" s="5" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
     </row>
     <row r="317" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A317" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B317" s="5" t="s">
-        <v>231</v>
+        <v>205</v>
       </c>
     </row>
     <row r="318" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A318" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B318" s="5" t="s">
-        <v>205</v>
+        <v>233</v>
       </c>
     </row>
     <row r="319" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A319" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B319" s="5" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="320" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A320" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B320" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="321" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A321" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B321" s="5" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
     <row r="322" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A322" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B322" s="5" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
     </row>
     <row r="323" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A323" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B323" s="5" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="324" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A324" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B324" s="5" t="s">
-        <v>238</v>
+        <v>314</v>
       </c>
     </row>
     <row r="325" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A325" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B325" s="5" t="s">
-        <v>314</v>
+        <v>378</v>
       </c>
     </row>
     <row r="326" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A326" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B326" s="5" t="s">
-        <v>378</v>
+        <v>220</v>
       </c>
     </row>
     <row r="327" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A327" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B327" s="5" t="s">
-        <v>220</v>
+        <v>441</v>
       </c>
     </row>
     <row r="328" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A328" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B328" s="5" t="s">
-        <v>441</v>
+        <v>330</v>
       </c>
     </row>
     <row r="329" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A329" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B329" s="5" t="s">
-        <v>330</v>
+        <v>442</v>
       </c>
     </row>
     <row r="330" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A330" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B330" s="5" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
     </row>
     <row r="331" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A331" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B331" s="5" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
     </row>
     <row r="332" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A332" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B332" s="5" t="s">
-        <v>444</v>
+        <v>470</v>
       </c>
     </row>
     <row r="333" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A333" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B333" s="5" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
     </row>
     <row r="334" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A334" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B334" s="5" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
     </row>
     <row r="335" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A335" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B335" s="5" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
     </row>
     <row r="336" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A336" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B336" s="5" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="337" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A337" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B337" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
     </row>
     <row r="338" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A338" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B338" s="5" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
     </row>
     <row r="339" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A339" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B339" s="5" t="s">
-        <v>479</v>
+        <v>331</v>
       </c>
     </row>
     <row r="340" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A340" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B340" s="5" t="s">
-        <v>331</v>
+        <v>477</v>
       </c>
     </row>
     <row r="341" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A341" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B341" s="5" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="342" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A342" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B342" s="5" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
     </row>
     <row r="343" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A343" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B343" s="5" t="s">
-        <v>482</v>
+        <v>223</v>
       </c>
     </row>
     <row r="344" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A344" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B344" s="5" t="s">
-        <v>223</v>
+        <v>480</v>
       </c>
     </row>
     <row r="345" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A345" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B345" s="5" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
     </row>
     <row r="346" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A346" s="1" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
       <c r="B346" s="5" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
     </row>
     <row r="347" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A347" s="1" t="s">
-        <v>486</v>
-      </c>
-      <c r="B347" s="5" t="s">
-        <v>485</v>
+        <v>520</v>
+      </c>
+      <c r="B347" s="7" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="348" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A348" s="1" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B348" s="7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="349" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A349" s="1" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B349" s="7" t="s">
-        <v>77</v>
+        <v>198</v>
       </c>
     </row>
     <row r="350" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A350" s="1" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B350" s="7" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="351" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A351" s="1" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B351" s="7" t="s">
-        <v>199</v>
+        <v>78</v>
       </c>
     </row>
     <row r="352" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A352" s="1" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B352" s="7" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="353" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A353" s="1" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B353" s="7" t="s">
-        <v>80</v>
+        <v>483</v>
       </c>
     </row>
     <row r="354" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A354" s="1" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B354" s="7" t="s">
-        <v>487</v>
+        <v>156</v>
       </c>
     </row>
     <row r="355" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A355" s="1" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B355" s="7" t="s">
-        <v>156</v>
+        <v>81</v>
       </c>
     </row>
     <row r="356" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A356" s="1" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B356" s="7" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="357" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A357" s="1" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B357" s="7" t="s">
-        <v>79</v>
+        <v>200</v>
       </c>
     </row>
     <row r="358" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A358" s="1" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B358" s="7" t="s">
-        <v>200</v>
+        <v>108</v>
       </c>
     </row>
     <row r="359" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A359" s="1" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B359" s="7" t="s">
-        <v>108</v>
+        <v>201</v>
       </c>
     </row>
     <row r="360" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A360" s="1" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B360" s="7" t="s">
-        <v>201</v>
+        <v>339</v>
       </c>
     </row>
     <row r="361" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A361" s="1" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B361" s="7" t="s">
-        <v>339</v>
+        <v>364</v>
       </c>
     </row>
     <row r="362" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A362" s="1" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B362" s="7" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="363" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A363" s="1" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B363" s="7" t="s">
-        <v>365</v>
+        <v>392</v>
       </c>
     </row>
     <row r="364" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A364" s="1" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B364" s="7" t="s">
-        <v>392</v>
+        <v>315</v>
       </c>
     </row>
     <row r="365" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A365" s="1" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B365" s="7" t="s">
-        <v>315</v>
+        <v>393</v>
       </c>
     </row>
     <row r="366" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A366" s="1" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B366" s="7" t="s">
-        <v>393</v>
+        <v>111</v>
       </c>
     </row>
     <row r="367" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A367" s="1" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B367" s="7" t="s">
-        <v>111</v>
+        <v>484</v>
       </c>
     </row>
     <row r="368" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A368" s="1" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B368" s="7" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
     </row>
     <row r="369" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A369" s="1" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B369" s="7" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
     </row>
     <row r="370" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A370" s="1" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B370" s="7" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
     </row>
     <row r="371" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A371" s="1" t="s">
-        <v>493</v>
-      </c>
-      <c r="B371" s="7" t="s">
-        <v>491</v>
+        <v>520</v>
+      </c>
+      <c r="B371" s="10" t="s">
+        <v>488</v>
       </c>
     </row>
     <row r="372" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A372" s="1" t="s">
-        <v>493</v>
-      </c>
-      <c r="B372" s="10" t="s">
-        <v>492</v>
+        <v>515</v>
+      </c>
+      <c r="B372" s="5" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="373" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A373" s="1" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
       <c r="B373" s="5" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
     </row>
     <row r="374" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A374" s="1" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
       <c r="B374" s="5" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
     </row>
     <row r="375" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A375" s="1" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
       <c r="B375" s="5" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
     </row>
     <row r="376" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A376" s="1" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
       <c r="B376" s="5" t="s">
-        <v>258</v>
+        <v>489</v>
       </c>
     </row>
     <row r="377" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A377" s="1" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
       <c r="B377" s="5" t="s">
-        <v>494</v>
+        <v>358</v>
       </c>
     </row>
     <row r="378" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A378" s="1" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
       <c r="B378" s="5" t="s">
-        <v>358</v>
+        <v>27</v>
       </c>
     </row>
     <row r="379" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A379" s="1" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
       <c r="B379" s="5" t="s">
-        <v>27</v>
+        <v>490</v>
       </c>
     </row>
     <row r="380" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A380" s="1" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
       <c r="B380" s="5" t="s">
-        <v>495</v>
+        <v>491</v>
       </c>
     </row>
     <row r="381" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A381" s="1" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
       <c r="B381" s="5" t="s">
-        <v>496</v>
+        <v>492</v>
       </c>
     </row>
     <row r="382" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A382" s="1" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
       <c r="B382" s="5" t="s">
-        <v>497</v>
+        <v>252</v>
       </c>
     </row>
     <row r="383" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A383" s="1" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
       <c r="B383" s="5" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="384" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A384" s="1" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
       <c r="B384" s="5" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="385" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A385" s="1" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
       <c r="B385" s="5" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
     </row>
     <row r="386" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A386" s="1" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
       <c r="B386" s="5" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="387" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A387" s="1" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
       <c r="B387" s="5" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
     </row>
     <row r="388" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A388" s="1" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
       <c r="B388" s="5" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
     </row>
     <row r="389" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A389" s="1" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
       <c r="B389" s="5" t="s">
-        <v>250</v>
+        <v>493</v>
       </c>
     </row>
     <row r="390" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A390" s="1" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
       <c r="B390" s="5" t="s">
-        <v>498</v>
+        <v>382</v>
       </c>
     </row>
     <row r="391" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A391" s="1" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
       <c r="B391" s="5" t="s">
-        <v>382</v>
+        <v>254</v>
       </c>
     </row>
     <row r="392" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A392" s="1" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
       <c r="B392" s="5" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
     </row>
     <row r="393" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A393" s="1" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
       <c r="B393" s="5" t="s">
-        <v>251</v>
+        <v>494</v>
       </c>
     </row>
     <row r="394" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A394" s="1" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
       <c r="B394" s="5" t="s">
-        <v>499</v>
+        <v>495</v>
       </c>
     </row>
     <row r="395" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A395" s="1" t="s">
-        <v>501</v>
+        <v>521</v>
       </c>
       <c r="B395" s="5" t="s">
-        <v>500</v>
+        <v>262</v>
       </c>
     </row>
     <row r="396" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A396" s="1" t="s">
-        <v>502</v>
+        <v>521</v>
       </c>
       <c r="B396" s="5" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="397" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A397" s="1" t="s">
-        <v>502</v>
+        <v>521</v>
       </c>
       <c r="B397" s="5" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="398" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A398" s="1" t="s">
-        <v>502</v>
+        <v>521</v>
       </c>
       <c r="B398" s="5" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
     </row>
     <row r="399" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A399" s="1" t="s">
-        <v>502</v>
+        <v>521</v>
       </c>
       <c r="B399" s="5" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
     </row>
     <row r="400" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A400" s="1" t="s">
-        <v>502</v>
+        <v>521</v>
       </c>
       <c r="B400" s="5" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="401" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A401" s="1" t="s">
-        <v>502</v>
+        <v>521</v>
       </c>
       <c r="B401" s="5" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="402" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A402" s="1" t="s">
-        <v>502</v>
+        <v>521</v>
       </c>
       <c r="B402" s="5" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="403" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A403" s="1" t="s">
-        <v>502</v>
+        <v>521</v>
       </c>
       <c r="B403" s="5" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="404" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A404" s="1" t="s">
-        <v>502</v>
+        <v>521</v>
       </c>
       <c r="B404" s="5" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="405" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A405" s="1" t="s">
-        <v>502</v>
+        <v>521</v>
       </c>
       <c r="B405" s="5" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="406" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A406" s="1" t="s">
-        <v>502</v>
+        <v>521</v>
       </c>
       <c r="B406" s="5" t="s">
-        <v>271</v>
+        <v>32</v>
       </c>
     </row>
     <row r="407" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A407" s="1" t="s">
-        <v>502</v>
+        <v>521</v>
       </c>
       <c r="B407" s="5" t="s">
-        <v>32</v>
+        <v>371</v>
       </c>
     </row>
     <row r="408" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A408" s="1" t="s">
-        <v>502</v>
+        <v>521</v>
       </c>
       <c r="B408" s="5" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
     </row>
     <row r="409" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A409" s="1" t="s">
-        <v>502</v>
+        <v>521</v>
       </c>
       <c r="B409" s="5" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
     </row>
     <row r="410" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A410" s="1" t="s">
-        <v>502</v>
+        <v>521</v>
       </c>
       <c r="B410" s="5" t="s">
-        <v>388</v>
+        <v>375</v>
       </c>
     </row>
     <row r="411" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A411" s="1" t="s">
-        <v>502</v>
+        <v>521</v>
       </c>
       <c r="B411" s="5" t="s">
-        <v>375</v>
+        <v>445</v>
       </c>
     </row>
     <row r="412" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A412" s="1" t="s">
-        <v>502</v>
+        <v>521</v>
       </c>
       <c r="B412" s="5" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
     </row>
     <row r="413" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A413" s="1" t="s">
-        <v>502</v>
+        <v>522</v>
       </c>
       <c r="B413" s="5" t="s">
-        <v>446</v>
+        <v>156</v>
       </c>
     </row>
     <row r="414" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A414" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B414" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="415" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A415" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B415" s="5" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="416" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A416" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B416" s="5" t="s">
-        <v>158</v>
+        <v>496</v>
       </c>
     </row>
     <row r="417" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A417" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B417" s="5" t="s">
-        <v>503</v>
+        <v>159</v>
       </c>
     </row>
     <row r="418" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A418" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B418" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="419" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A419" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B419" s="5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="420" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A420" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B420" s="5" t="s">
-        <v>161</v>
+        <v>183</v>
       </c>
     </row>
     <row r="421" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A421" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B421" s="5" t="s">
-        <v>183</v>
+        <v>162</v>
       </c>
     </row>
     <row r="422" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A422" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B422" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="423" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A423" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B423" s="5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="424" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A424" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B424" s="5" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="425" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A425" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B425" s="5" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
     </row>
     <row r="426" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A426" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B426" s="5" t="s">
-        <v>119</v>
+        <v>166</v>
       </c>
     </row>
     <row r="427" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A427" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B427" s="5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="428" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A428" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B428" s="5" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="429" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A429" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B429" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="430" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A430" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B430" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="431" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A431" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B431" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="432" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A432" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B432" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="433" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A433" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B433" s="5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="434" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A434" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B434" s="5" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="435" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A435" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B435" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="436" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A436" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B436" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="437" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A437" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B437" s="5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="438" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A438" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B438" s="5" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="439" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A439" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B439" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="440" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A440" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B440" s="5" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="441" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A441" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B441" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="442" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A442" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B442" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="443" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A443" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B443" s="5" t="s">
-        <v>182</v>
+        <v>367</v>
       </c>
     </row>
     <row r="444" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A444" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B444" s="5" t="s">
-        <v>367</v>
+        <v>421</v>
       </c>
     </row>
     <row r="445" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A445" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B445" s="5" t="s">
-        <v>421</v>
+        <v>497</v>
       </c>
     </row>
     <row r="446" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A446" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B446" s="5" t="s">
-        <v>504</v>
+        <v>447</v>
       </c>
     </row>
     <row r="447" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A447" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B447" s="5" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="448" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A448" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B448" s="5" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
     </row>
     <row r="449" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A449" s="1" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B449" s="5" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="450" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A450" s="1" t="s">
-        <v>505</v>
+        <v>513</v>
       </c>
       <c r="B450" s="5" t="s">
-        <v>450</v>
+        <v>108</v>
       </c>
     </row>
     <row r="451" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A451" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B451" s="5" t="s">
-        <v>27</v>
+        <v>109</v>
       </c>
     </row>
     <row r="452" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A452" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B452" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="453" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A453" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B453" s="5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="454" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A454" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B454" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="455" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A455" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B455" s="5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="456" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A456" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B456" s="5" t="s">
-        <v>112</v>
+        <v>346</v>
       </c>
     </row>
     <row r="457" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A457" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B457" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="458" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A458" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B458" s="5" t="s">
-        <v>346</v>
+        <v>115</v>
       </c>
     </row>
     <row r="459" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A459" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B459" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="460" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A460" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B460" s="5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="461" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A461" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B461" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="462" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A462" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B462" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="463" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A463" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B463" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="464" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A464" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B464" s="5" t="s">
-        <v>119</v>
+        <v>80</v>
       </c>
     </row>
     <row r="465" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A465" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B465" s="5" t="s">
-        <v>120</v>
+        <v>101</v>
       </c>
     </row>
     <row r="466" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A466" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B466" s="5" t="s">
-        <v>80</v>
+        <v>121</v>
       </c>
     </row>
     <row r="467" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A467" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B467" s="5" t="s">
-        <v>101</v>
+        <v>123</v>
       </c>
     </row>
     <row r="468" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A468" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B468" s="5" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="469" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A469" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B469" s="5" t="s">
-        <v>123</v>
+        <v>139</v>
       </c>
     </row>
     <row r="470" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A470" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B470" s="5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="471" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A471" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B471" s="5" t="s">
-        <v>139</v>
+        <v>26</v>
       </c>
     </row>
     <row r="472" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A472" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B472" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="473" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A473" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B473" s="5" t="s">
-        <v>26</v>
+        <v>140</v>
       </c>
     </row>
     <row r="474" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A474" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B474" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="475" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A475" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B475" s="5" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
     </row>
     <row r="476" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A476" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B476" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="477" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A477" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B477" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="478" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A478" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B478" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="479" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A479" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B479" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="480" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A480" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B480" s="5" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="481" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A481" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B481" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="482" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A482" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B482" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
     </row>
     <row r="483" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A483" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B483" s="5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="484" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A484" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B484" s="5" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
     </row>
     <row r="485" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A485" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B485" s="5" t="s">
-        <v>135</v>
+        <v>122</v>
       </c>
     </row>
     <row r="486" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A486" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B486" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="487" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A487" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B487" s="5" t="s">
-        <v>122</v>
+        <v>138</v>
       </c>
     </row>
     <row r="488" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A488" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B488" s="5" t="s">
-        <v>137</v>
+        <v>362</v>
       </c>
     </row>
     <row r="489" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A489" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B489" s="5" t="s">
-        <v>138</v>
+        <v>390</v>
       </c>
     </row>
     <row r="490" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A490" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B490" s="5" t="s">
-        <v>362</v>
+        <v>498</v>
       </c>
     </row>
     <row r="491" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A491" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B491" s="5" t="s">
-        <v>390</v>
+        <v>499</v>
       </c>
     </row>
     <row r="492" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A492" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B492" s="5" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
     </row>
     <row r="493" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A493" s="1" t="s">
-        <v>509</v>
+        <v>516</v>
       </c>
       <c r="B493" s="5" t="s">
-        <v>507</v>
+        <v>184</v>
       </c>
     </row>
     <row r="494" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A494" s="1" t="s">
-        <v>509</v>
+        <v>516</v>
       </c>
       <c r="B494" s="5" t="s">
-        <v>508</v>
+        <v>188</v>
       </c>
     </row>
     <row r="495" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A495" s="1" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B495" s="5" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="496" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A496" s="1" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B496" s="5" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
     <row r="497" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A497" s="1" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B497" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="498" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A498" s="1" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B498" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="499" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A499" s="1" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B499" s="5" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="500" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A500" s="1" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B500" s="5" t="s">
-        <v>186</v>
+        <v>501</v>
       </c>
     </row>
     <row r="501" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A501" s="1" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B501" s="5" t="s">
-        <v>187</v>
+        <v>502</v>
       </c>
     </row>
     <row r="502" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A502" s="1" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B502" s="5" t="s">
-        <v>510</v>
+        <v>503</v>
       </c>
     </row>
     <row r="503" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A503" s="1" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B503" s="5" t="s">
-        <v>511</v>
+        <v>504</v>
       </c>
     </row>
     <row r="504" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A504" s="1" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B504" s="5" t="s">
-        <v>512</v>
+        <v>505</v>
       </c>
     </row>
     <row r="505" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A505" s="1" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B505" s="5" t="s">
-        <v>513</v>
+        <v>506</v>
       </c>
     </row>
     <row r="506" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A506" s="1" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B506" s="5" t="s">
-        <v>514</v>
+        <v>507</v>
       </c>
     </row>
     <row r="507" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A507" s="1" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B507" s="5" t="s">
-        <v>515</v>
+        <v>273</v>
       </c>
     </row>
     <row r="508" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A508" s="1" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B508" s="5" t="s">
-        <v>516</v>
+        <v>288</v>
       </c>
     </row>
     <row r="509" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A509" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B509" s="5" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="510" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A510" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B510" s="5" t="s">
-        <v>288</v>
+        <v>275</v>
       </c>
     </row>
     <row r="511" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A511" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B511" s="5" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="512" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A512" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B512" s="5" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
     <row r="513" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A513" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B513" s="5" t="s">
-        <v>276</v>
+        <v>36</v>
       </c>
     </row>
     <row r="514" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A514" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B514" s="5" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="515" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A515" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B515" s="5" t="s">
-        <v>36</v>
+        <v>279</v>
       </c>
     </row>
     <row r="516" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A516" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B516" s="5" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="517" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A517" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B517" s="5" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="518" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A518" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B518" s="5" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="519" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A519" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B519" s="5" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="520" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A520" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B520" s="5" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="521" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A521" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B521" s="5" t="s">
-        <v>283</v>
+        <v>451</v>
       </c>
     </row>
     <row r="522" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A522" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B522" s="5" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="523" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A523" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B523" s="5" t="s">
-        <v>451</v>
+        <v>286</v>
       </c>
     </row>
     <row r="524" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A524" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B524" s="5" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="525" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A525" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B525" s="5" t="s">
-        <v>286</v>
+        <v>131</v>
       </c>
     </row>
     <row r="526" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A526" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B526" s="5" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="527" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A527" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B527" s="5" t="s">
-        <v>131</v>
+        <v>290</v>
       </c>
     </row>
     <row r="528" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A528" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B528" s="5" t="s">
-        <v>289</v>
+        <v>195</v>
       </c>
     </row>
     <row r="529" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A529" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B529" s="5" t="s">
-        <v>290</v>
+        <v>9</v>
       </c>
     </row>
     <row r="530" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A530" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B530" s="5" t="s">
-        <v>195</v>
+        <v>291</v>
       </c>
     </row>
     <row r="531" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A531" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B531" s="5" t="s">
-        <v>9</v>
+        <v>192</v>
       </c>
     </row>
     <row r="532" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A532" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B532" s="5" t="s">
-        <v>291</v>
+        <v>454</v>
       </c>
     </row>
     <row r="533" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A533" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B533" s="5" t="s">
-        <v>192</v>
+        <v>292</v>
       </c>
     </row>
     <row r="534" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A534" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B534" s="5" t="s">
-        <v>454</v>
+        <v>293</v>
       </c>
     </row>
     <row r="535" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A535" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B535" s="5" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="536" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A536" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B536" s="5" t="s">
-        <v>293</v>
+        <v>452</v>
       </c>
     </row>
     <row r="537" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A537" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B537" s="5" t="s">
-        <v>294</v>
+        <v>508</v>
       </c>
     </row>
     <row r="538" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A538" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B538" s="5" t="s">
-        <v>452</v>
+        <v>295</v>
       </c>
     </row>
     <row r="539" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A539" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B539" s="5" t="s">
-        <v>518</v>
+        <v>455</v>
       </c>
     </row>
     <row r="540" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A540" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B540" s="5" t="s">
-        <v>295</v>
+        <v>360</v>
       </c>
     </row>
     <row r="541" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A541" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B541" s="5" t="s">
-        <v>455</v>
+        <v>370</v>
       </c>
     </row>
     <row r="542" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A542" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B542" s="5" t="s">
-        <v>360</v>
+        <v>376</v>
       </c>
     </row>
     <row r="543" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A543" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B543" s="5" t="s">
-        <v>370</v>
+        <v>453</v>
       </c>
     </row>
     <row r="544" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
@@ -6337,7 +6337,7 @@
         <v>519</v>
       </c>
       <c r="B544" s="5" t="s">
-        <v>376</v>
+        <v>142</v>
       </c>
     </row>
     <row r="545" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
@@ -6345,182 +6345,166 @@
         <v>519</v>
       </c>
       <c r="B545" s="5" t="s">
-        <v>453</v>
+        <v>143</v>
       </c>
     </row>
     <row r="546" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A546" s="1" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="B546" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="547" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A547" s="1" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="B547" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="548" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A548" s="1" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="B548" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="549" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A549" s="1" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="B549" s="5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="550" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A550" s="1" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="B550" s="5" t="s">
-        <v>146</v>
+        <v>345</v>
       </c>
     </row>
     <row r="551" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A551" s="1" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="B551" s="5" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
     </row>
     <row r="552" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A552" s="1" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="B552" s="5" t="s">
-        <v>345</v>
+        <v>155</v>
       </c>
     </row>
     <row r="553" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A553" s="1" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="B553" s="5" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
     </row>
     <row r="554" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A554" s="1" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="B554" s="5" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
     </row>
     <row r="555" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A555" s="1" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="B555" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="556" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A556" s="1" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="B556" s="5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="557" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A557" s="1" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="B557" s="5" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="558" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A558" s="1" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="B558" s="5" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="559" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A559" s="1" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="B559" s="5" t="s">
-        <v>152</v>
+        <v>375</v>
       </c>
     </row>
     <row r="560" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A560" s="1" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="B560" s="5" t="s">
-        <v>153</v>
+        <v>420</v>
       </c>
     </row>
     <row r="561" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A561" s="1" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="B561" s="5" t="s">
-        <v>375</v>
+        <v>456</v>
       </c>
     </row>
     <row r="562" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A562" s="1" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="B562" s="5" t="s">
-        <v>420</v>
+        <v>457</v>
       </c>
     </row>
     <row r="563" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A563" s="1" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="B563" s="5" t="s">
-        <v>456</v>
+        <v>509</v>
       </c>
     </row>
     <row r="564" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A564" s="1" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="B564" s="5" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="565" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A565" s="1" t="s">
-        <v>522</v>
-      </c>
-      <c r="B565" s="5" t="s">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="566" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A566" s="1" t="s">
-        <v>522</v>
-      </c>
-      <c r="B566" s="5" t="s">
-        <v>521</v>
+        <v>510</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B566" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <autoFilter ref="A1:B564" xr:uid="{00000000-0001-0000-0100-000000000000}">
     <filterColumn colId="0">
       <filters>
-        <filter val="Crosyen"/>
+        <filter val="tropecos"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>